<commit_message>
streamlit UI complete and working - metrics displaying correctly - full pipeline end to end
</commit_message>
<xml_diff>
--- a/data/output-data/chc_report.xlsx
+++ b/data/output-data/chc_report.xlsx
@@ -1144,113 +1144,113 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>CHC-PT00007-2023-05-08</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>PT00007</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>MRN+DATE</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="4" t="n">
         <v>158</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>CYT-59615</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="5" t="n">
         <v>45054</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>HSIL. Features consistent with CIN 2-3. Colposcopy recommended.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Unsatisfactory</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>SP-86106</t>
         </is>
       </c>
-      <c r="K7" s="3" t="n">
+      <c r="K7" s="5" t="n">
         <v>45212</v>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Cervical intraepithelial neoplasia, grade 1 (CIN 1/LSIL).</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>ECC</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>HSIL</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>HSIL</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="R7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="S7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T7" s="2" t="inlineStr">
-        <is>
-          <t>minor_discordant</t>
-        </is>
-      </c>
-      <c r="U7" s="2" t="inlineStr">
-        <is>
-          <t>minor_overcall</t>
-        </is>
-      </c>
-      <c r="V7" s="2" t="inlineStr">
-        <is>
-          <t>overcall</t>
-        </is>
-      </c>
-      <c r="W7" s="2" t="inlineStr">
-        <is>
-          <t>minor</t>
-        </is>
-      </c>
-      <c r="X7" s="2" t="inlineStr">
-        <is>
-          <t>HSIL→LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="Y7" s="2" t="b">
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>concordant</t>
+        </is>
+      </c>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>exact_agreement</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="W7" s="4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="X7" s="4" t="inlineStr">
+        <is>
+          <t>HSIL→HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="Y7" s="4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="R10" s="2" t="b">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>LSIL→HSIL (CIN3)</t>
+          <t>LSIL→HSIL (CIN2)</t>
         </is>
       </c>
       <c r="Y10" s="2" t="b">
@@ -1921,113 +1921,113 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>CHC-PT00015-2024-01-06</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>PT00015</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>MRN+DATE</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="4" t="n">
         <v>93</v>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>CYT-38746</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="5" t="n">
         <v>45297</v>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>HIGH GRADE SQUAMOUS INTRAEPITHELIAL LESION (HSIL)</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Adequate</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>SP-39041</t>
         </is>
       </c>
-      <c r="K14" s="3" t="n">
+      <c r="K14" s="5" t="n">
         <v>45390</v>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Cervical intraepithelial neoplasia, grade 1 (CIN 1/LSIL).</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Cervical biopsy</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>HSIL</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>HSIL</t>
         </is>
       </c>
-      <c r="Q14" s="2" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="R14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="S14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T14" s="2" t="inlineStr">
-        <is>
-          <t>minor_discordant</t>
-        </is>
-      </c>
-      <c r="U14" s="2" t="inlineStr">
-        <is>
-          <t>minor_overcall</t>
-        </is>
-      </c>
-      <c r="V14" s="2" t="inlineStr">
-        <is>
-          <t>overcall</t>
-        </is>
-      </c>
-      <c r="W14" s="2" t="inlineStr">
-        <is>
-          <t>minor</t>
-        </is>
-      </c>
-      <c r="X14" s="2" t="inlineStr">
-        <is>
-          <t>HSIL→LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="Y14" s="2" t="b">
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="R14" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S14" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>concordant</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="inlineStr">
+        <is>
+          <t>exact_agreement</t>
+        </is>
+      </c>
+      <c r="V14" s="4" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="W14" s="4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="X14" s="4" t="inlineStr">
+        <is>
+          <t>HSIL→HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="Y14" s="4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>AGC-ECX/EMC NEO</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>AGC-ECX/EMC NEO</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="Q15" s="4" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="X15" s="4" t="inlineStr">
         <is>
-          <t>AGC-ECX/EMC NEO→Adenocarcinoma</t>
+          <t>AGC-NEO→Adenocarcinoma</t>
         </is>
       </c>
       <c r="Y15" s="4" t="b">
@@ -3031,113 +3031,113 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>CHC-PT00026-2023-03-07</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>PT00026</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>MRN+DATE</t>
         </is>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D24" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>CYT-54313</t>
         </is>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="3" t="n">
         <v>44992</v>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>High grade squamous intraepithelial lesion. Cannot exclude invasion.</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Satisfactory for evaluation</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>SP-88966</t>
         </is>
       </c>
-      <c r="K24" s="5" t="n">
+      <c r="K24" s="3" t="n">
         <v>45049</v>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>High grade CIN (CIN 2-3). Cannot exclude early invasion.</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Cervical biopsy</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t>HSIL</t>
-        </is>
-      </c>
-      <c r="O24" s="4" t="inlineStr">
-        <is>
-          <t>HSIL (CIN3)</t>
-        </is>
-      </c>
-      <c r="P24" s="4" t="inlineStr">
-        <is>
-          <t>HSIL</t>
-        </is>
-      </c>
-      <c r="Q24" s="4" t="inlineStr">
-        <is>
-          <t>HSIL (CIN3)</t>
-        </is>
-      </c>
-      <c r="R24" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="S24" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="T24" s="4" t="inlineStr">
-        <is>
-          <t>concordant</t>
-        </is>
-      </c>
-      <c r="U24" s="4" t="inlineStr">
-        <is>
-          <t>exact_agreement</t>
-        </is>
-      </c>
-      <c r="V24" s="4" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="W24" s="4" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="X24" s="4" t="inlineStr">
-        <is>
-          <t>HSIL→HSIL (CIN3)</t>
-        </is>
-      </c>
-      <c r="Y24" s="4" t="b">
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>minor_discordant</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>minor_overcall</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>overcall</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT→HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="Q27" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="R27" s="6" t="b">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="X27" s="6" t="inlineStr">
         <is>
-          <t>NILM→HSIL (CIN3)</t>
+          <t>NILM→HSIL (CIN2)</t>
         </is>
       </c>
       <c r="Y27" s="6" t="b">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="O38" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="P38" s="6" t="inlineStr">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="Q38" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="R38" s="6" t="b">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="X38" s="6" t="inlineStr">
         <is>
-          <t>NILM→HSIL (CIN3)</t>
+          <t>NILM→HSIL (CIN2)</t>
         </is>
       </c>
       <c r="Y38" s="6" t="b">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="R42" s="2" t="b">
@@ -5132,7 +5132,7 @@
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
-          <t>ASC-US→HSIL (CIN3)</t>
+          <t>ASC-US→HSIL (CIN2)</t>
         </is>
       </c>
       <c r="Y42" s="2" t="b">
@@ -6028,113 +6028,113 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>CHC-PT00056-2023-04-21</t>
         </is>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>PT00056</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>MRN+DATE</t>
         </is>
       </c>
-      <c r="D51" s="6" t="n">
+      <c r="D51" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>CYT-60140</t>
         </is>
       </c>
-      <c r="F51" s="7" t="n">
+      <c r="F51" s="3" t="n">
         <v>45037</v>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>Positive for malignancy. Adenocarcinoma cannot be excluded.</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Adequate</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr"/>
-      <c r="J51" s="6" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
         <is>
           <t>SP-90356</t>
         </is>
       </c>
-      <c r="K51" s="7" t="n">
+      <c r="K51" s="3" t="n">
         <v>45127</v>
       </c>
-      <c r="L51" s="6" t="inlineStr">
+      <c r="L51" s="2" t="inlineStr">
         <is>
           <t>Cervical intraepithelial neoplasia, grade 1 (CIN 1/LSIL).</t>
         </is>
       </c>
-      <c r="M51" s="6" t="inlineStr">
+      <c r="M51" s="2" t="inlineStr">
         <is>
           <t>LEEP</t>
         </is>
       </c>
-      <c r="N51" s="6" t="inlineStr">
+      <c r="N51" s="2" t="inlineStr">
         <is>
           <t>MALIGNANT</t>
         </is>
       </c>
-      <c r="O51" s="6" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="P51" s="6" t="inlineStr">
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
         <is>
           <t>MALIGNANT</t>
         </is>
       </c>
-      <c r="Q51" s="6" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="R51" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="S51" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="T51" s="6" t="inlineStr">
-        <is>
-          <t>major_discordant</t>
-        </is>
-      </c>
-      <c r="U51" s="6" t="inlineStr">
-        <is>
-          <t>major_overcall</t>
-        </is>
-      </c>
-      <c r="V51" s="6" t="inlineStr">
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S51" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>minor_discordant</t>
+        </is>
+      </c>
+      <c r="U51" s="2" t="inlineStr">
+        <is>
+          <t>minor_overcall</t>
+        </is>
+      </c>
+      <c r="V51" s="2" t="inlineStr">
         <is>
           <t>overcall</t>
         </is>
       </c>
-      <c r="W51" s="6" t="inlineStr">
-        <is>
-          <t>major</t>
-        </is>
-      </c>
-      <c r="X51" s="6" t="inlineStr">
-        <is>
-          <t>MALIGNANT→LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="Y51" s="6" t="b">
+      <c r="W51" s="2" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT→HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="Y51" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="O61" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="P61" s="6" t="inlineStr">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="Q61" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="R61" s="6" t="b">
@@ -7241,7 +7241,7 @@
       </c>
       <c r="X61" s="6" t="inlineStr">
         <is>
-          <t>NILM→HSIL (CIN3)</t>
+          <t>NILM→HSIL (CIN2)</t>
         </is>
       </c>
       <c r="Y61" s="6" t="b">
@@ -8638,7 +8638,7 @@
       </c>
       <c r="N74" s="4" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="O74" s="4" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="P74" s="4" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="Q74" s="4" t="inlineStr">
@@ -8684,7 +8684,7 @@
       </c>
       <c r="X74" s="4" t="inlineStr">
         <is>
-          <t>ASC-US→LSIL (CIN1)</t>
+          <t>AGC→LSIL (CIN1)</t>
         </is>
       </c>
       <c r="Y74" s="4" t="b">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="O76" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="P76" s="6" t="inlineStr">
@@ -8875,7 +8875,7 @@
       </c>
       <c r="Q76" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="R76" s="6" t="b">
@@ -8906,7 +8906,7 @@
       </c>
       <c r="X76" s="6" t="inlineStr">
         <is>
-          <t>NILM→HSIL (CIN3)</t>
+          <t>NILM→HSIL (CIN2)</t>
         </is>
       </c>
       <c r="Y76" s="6" t="b">
@@ -9082,7 +9082,7 @@
       </c>
       <c r="N78" s="6" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="O78" s="6" t="inlineStr">
@@ -9092,7 +9092,7 @@
       </c>
       <c r="P78" s="6" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="Q78" s="6" t="inlineStr">
@@ -9128,7 +9128,7 @@
       </c>
       <c r="X78" s="6" t="inlineStr">
         <is>
-          <t>HSIL→Benign / Inflammatory (Negative)</t>
+          <t>MALIGNANT→Benign / Inflammatory (Negative)</t>
         </is>
       </c>
       <c r="Y78" s="6" t="b">
@@ -10197,7 +10197,7 @@
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="P88" s="2" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="Q88" s="2" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="R88" s="2" t="b">
@@ -10238,7 +10238,7 @@
       </c>
       <c r="X88" s="2" t="inlineStr">
         <is>
-          <t>ASC-US→HSIL (CIN3)</t>
+          <t>ASC-US→HSIL (CIN2)</t>
         </is>
       </c>
       <c r="Y88" s="2" t="b">
@@ -10357,224 +10357,224 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="4" t="inlineStr">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>CHC-PT00103-2024-05-10</t>
         </is>
       </c>
-      <c r="B90" s="4" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>PT00103</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>MRN+DATE</t>
         </is>
       </c>
-      <c r="D90" s="4" t="n">
+      <c r="D90" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="E90" s="2" t="inlineStr">
         <is>
           <t>CYT-46241</t>
         </is>
       </c>
-      <c r="F90" s="5" t="n">
+      <c r="F90" s="3" t="n">
         <v>45422</v>
       </c>
-      <c r="G90" s="4" t="inlineStr">
+      <c r="G90" s="2" t="inlineStr">
         <is>
           <t>High grade squamous intraepithelial lesion. Cannot exclude invasion.</t>
         </is>
       </c>
-      <c r="H90" s="4" t="inlineStr">
+      <c r="H90" s="2" t="inlineStr">
         <is>
           <t>Unsatisfactory</t>
         </is>
       </c>
-      <c r="I90" s="4" t="inlineStr"/>
-      <c r="J90" s="4" t="inlineStr">
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr">
         <is>
           <t>SP-67104</t>
         </is>
       </c>
-      <c r="K90" s="5" t="n">
+      <c r="K90" s="3" t="n">
         <v>45491</v>
       </c>
-      <c r="L90" s="4" t="inlineStr">
+      <c r="L90" s="2" t="inlineStr">
         <is>
           <t>High grade CIN (CIN 2-3). Cannot exclude early invasion.</t>
         </is>
       </c>
-      <c r="M90" s="4" t="inlineStr">
+      <c r="M90" s="2" t="inlineStr">
         <is>
           <t>Cervical biopsy</t>
         </is>
       </c>
-      <c r="N90" s="4" t="inlineStr">
-        <is>
-          <t>HSIL</t>
-        </is>
-      </c>
-      <c r="O90" s="4" t="inlineStr">
-        <is>
-          <t>HSIL (CIN3)</t>
-        </is>
-      </c>
-      <c r="P90" s="4" t="inlineStr">
-        <is>
-          <t>HSIL</t>
-        </is>
-      </c>
-      <c r="Q90" s="4" t="inlineStr">
-        <is>
-          <t>HSIL (CIN3)</t>
-        </is>
-      </c>
-      <c r="R90" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="S90" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="T90" s="4" t="inlineStr">
-        <is>
-          <t>concordant</t>
-        </is>
-      </c>
-      <c r="U90" s="4" t="inlineStr">
-        <is>
-          <t>exact_agreement</t>
-        </is>
-      </c>
-      <c r="V90" s="4" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="W90" s="4" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="X90" s="4" t="inlineStr">
-        <is>
-          <t>HSIL→HSIL (CIN3)</t>
-        </is>
-      </c>
-      <c r="Y90" s="4" t="b">
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT</t>
+        </is>
+      </c>
+      <c r="Q90" s="2" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="R90" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S90" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T90" s="2" t="inlineStr">
+        <is>
+          <t>minor_discordant</t>
+        </is>
+      </c>
+      <c r="U90" s="2" t="inlineStr">
+        <is>
+          <t>minor_overcall</t>
+        </is>
+      </c>
+      <c r="V90" s="2" t="inlineStr">
+        <is>
+          <t>overcall</t>
+        </is>
+      </c>
+      <c r="W90" s="2" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="X90" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT→HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="Y90" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="4" t="inlineStr">
+      <c r="A91" s="2" t="inlineStr">
         <is>
           <t>CHC-PT00104-2023-08-21</t>
         </is>
       </c>
-      <c r="B91" s="4" t="inlineStr">
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>PT00104</t>
         </is>
       </c>
-      <c r="C91" s="4" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>MRN+DATE</t>
         </is>
       </c>
-      <c r="D91" s="4" t="n">
+      <c r="D91" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E91" s="4" t="inlineStr">
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>CYT-57301</t>
         </is>
       </c>
-      <c r="F91" s="5" t="n">
+      <c r="F91" s="3" t="n">
         <v>45159</v>
       </c>
-      <c r="G91" s="4" t="inlineStr">
+      <c r="G91" s="2" t="inlineStr">
         <is>
           <t>ASC-US. Cannot exclude low grade squamous intraepithelial lesion.</t>
         </is>
       </c>
-      <c r="H91" s="4" t="inlineStr">
+      <c r="H91" s="2" t="inlineStr">
         <is>
           <t>Satisfactory</t>
         </is>
       </c>
-      <c r="I91" s="4" t="inlineStr"/>
-      <c r="J91" s="4" t="inlineStr">
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr">
         <is>
           <t>SP-75193</t>
         </is>
       </c>
-      <c r="K91" s="5" t="n">
+      <c r="K91" s="3" t="n">
         <v>45167</v>
       </c>
-      <c r="L91" s="4" t="inlineStr">
+      <c r="L91" s="2" t="inlineStr">
         <is>
           <t>Cervical intraepithelial neoplasia, grade 1 (CIN 1/LSIL).</t>
         </is>
       </c>
-      <c r="M91" s="4" t="inlineStr">
+      <c r="M91" s="2" t="inlineStr">
         <is>
           <t>Punch biopsy</t>
         </is>
       </c>
-      <c r="N91" s="4" t="inlineStr">
+      <c r="N91" s="2" t="inlineStr">
         <is>
           <t>ASC-US</t>
         </is>
       </c>
-      <c r="O91" s="4" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="P91" s="4" t="inlineStr">
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="P91" s="2" t="inlineStr">
         <is>
           <t>ASC-US</t>
         </is>
       </c>
-      <c r="Q91" s="4" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="R91" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="S91" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="T91" s="4" t="inlineStr">
-        <is>
-          <t>concordant</t>
-        </is>
-      </c>
-      <c r="U91" s="4" t="inlineStr">
-        <is>
-          <t>exact_agreement</t>
-        </is>
-      </c>
-      <c r="V91" s="4" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="W91" s="4" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="X91" s="4" t="inlineStr">
-        <is>
-          <t>ASC-US→LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="Y91" s="4" t="b">
+      <c r="Q91" s="2" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="R91" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S91" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T91" s="2" t="inlineStr">
+        <is>
+          <t>minor_discordant</t>
+        </is>
+      </c>
+      <c r="U91" s="2" t="inlineStr">
+        <is>
+          <t>minor_undercall</t>
+        </is>
+      </c>
+      <c r="V91" s="2" t="inlineStr">
+        <is>
+          <t>undercall</t>
+        </is>
+      </c>
+      <c r="W91" s="2" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="X91" s="2" t="inlineStr">
+        <is>
+          <t>ASC-US→HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="Y91" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -11578,113 +11578,113 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="inlineStr">
+      <c r="A101" s="4" t="inlineStr">
         <is>
           <t>CHC-PT00114-2023-10-17</t>
         </is>
       </c>
-      <c r="B101" s="2" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>PT00114</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr">
+      <c r="C101" s="4" t="inlineStr">
         <is>
           <t>MRN+DATE</t>
         </is>
       </c>
-      <c r="D101" s="2" t="n">
+      <c r="D101" s="4" t="n">
         <v>139</v>
       </c>
-      <c r="E101" s="2" t="inlineStr">
+      <c r="E101" s="4" t="inlineStr">
         <is>
           <t>CYT-69510</t>
         </is>
       </c>
-      <c r="F101" s="3" t="n">
+      <c r="F101" s="5" t="n">
         <v>45216</v>
       </c>
-      <c r="G101" s="2" t="inlineStr">
+      <c r="G101" s="4" t="inlineStr">
         <is>
           <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
         </is>
       </c>
-      <c r="H101" s="2" t="inlineStr">
+      <c r="H101" s="4" t="inlineStr">
         <is>
           <t>Satisfactory for evaluation</t>
         </is>
       </c>
-      <c r="I101" s="2" t="inlineStr"/>
-      <c r="J101" s="2" t="inlineStr">
+      <c r="I101" s="4" t="inlineStr"/>
+      <c r="J101" s="4" t="inlineStr">
         <is>
           <t>SP-30056</t>
         </is>
       </c>
-      <c r="K101" s="3" t="n">
+      <c r="K101" s="5" t="n">
         <v>45355</v>
       </c>
-      <c r="L101" s="2" t="inlineStr">
+      <c r="L101" s="4" t="inlineStr">
         <is>
           <t>Cervical intraepithelial neoplasia, grade 1 (CIN 1/LSIL).</t>
         </is>
       </c>
-      <c r="M101" s="2" t="inlineStr">
+      <c r="M101" s="4" t="inlineStr">
         <is>
           <t>Punch biopsy</t>
         </is>
       </c>
-      <c r="N101" s="2" t="inlineStr">
+      <c r="N101" s="4" t="inlineStr">
         <is>
           <t>ASC-H</t>
         </is>
       </c>
-      <c r="O101" s="2" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="P101" s="2" t="inlineStr">
+      <c r="O101" s="4" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="P101" s="4" t="inlineStr">
         <is>
           <t>ASC-H</t>
         </is>
       </c>
-      <c r="Q101" s="2" t="inlineStr">
-        <is>
-          <t>LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="R101" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="S101" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T101" s="2" t="inlineStr">
-        <is>
-          <t>minor_discordant</t>
-        </is>
-      </c>
-      <c r="U101" s="2" t="inlineStr">
-        <is>
-          <t>minor_overcall</t>
-        </is>
-      </c>
-      <c r="V101" s="2" t="inlineStr">
-        <is>
-          <t>overcall</t>
-        </is>
-      </c>
-      <c r="W101" s="2" t="inlineStr">
-        <is>
-          <t>minor</t>
-        </is>
-      </c>
-      <c r="X101" s="2" t="inlineStr">
-        <is>
-          <t>ASC-H→LSIL (CIN1)</t>
-        </is>
-      </c>
-      <c r="Y101" s="2" t="b">
+      <c r="Q101" s="4" t="inlineStr">
+        <is>
+          <t>HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="R101" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S101" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="T101" s="4" t="inlineStr">
+        <is>
+          <t>concordant</t>
+        </is>
+      </c>
+      <c r="U101" s="4" t="inlineStr">
+        <is>
+          <t>exact_agreement</t>
+        </is>
+      </c>
+      <c r="V101" s="4" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="W101" s="4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="X101" s="4" t="inlineStr">
+        <is>
+          <t>ASC-H→HSIL (CIN2)</t>
+        </is>
+      </c>
+      <c r="Y101" s="4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -11857,7 +11857,7 @@
       </c>
       <c r="N103" s="2" t="inlineStr">
         <is>
-          <t>AGC-ECX/EMC NEO</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="O103" s="2" t="inlineStr">
@@ -11867,7 +11867,7 @@
       </c>
       <c r="P103" s="2" t="inlineStr">
         <is>
-          <t>AGC-ECX/EMC NEO</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="Q103" s="2" t="inlineStr">
@@ -11903,7 +11903,7 @@
       </c>
       <c r="X103" s="2" t="inlineStr">
         <is>
-          <t>AGC-ECX/EMC NEO→LSIL (CIN1)</t>
+          <t>AGC-NEO→LSIL (CIN1)</t>
         </is>
       </c>
       <c r="Y103" s="2" t="b">
@@ -12133,113 +12133,113 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="4" t="inlineStr">
+      <c r="A106" s="2" t="inlineStr">
         <is>
           <t>CHC-PT00119-2023-08-23</t>
         </is>
       </c>
-      <c r="B106" s="4" t="inlineStr">
+      <c r="B106" s="2" t="inlineStr">
         <is>
           <t>PT00119</t>
         </is>
       </c>
-      <c r="C106" s="4" t="inlineStr">
+      <c r="C106" s="2" t="inlineStr">
         <is>
           <t>MRN+DATE</t>
         </is>
       </c>
-      <c r="D106" s="4" t="n">
+      <c r="D106" s="2" t="n">
         <v>134</v>
       </c>
-      <c r="E106" s="4" t="inlineStr">
+      <c r="E106" s="2" t="inlineStr">
         <is>
           <t>CYT-98381</t>
         </is>
       </c>
-      <c r="F106" s="5" t="n">
+      <c r="F106" s="3" t="n">
         <v>45161</v>
       </c>
-      <c r="G106" s="4" t="inlineStr">
+      <c r="G106" s="2" t="inlineStr">
         <is>
           <t>High grade squamous intraepithelial lesion. Cannot exclude invasion.</t>
         </is>
       </c>
-      <c r="H106" s="4" t="inlineStr">
+      <c r="H106" s="2" t="inlineStr">
         <is>
           <t>Satisfactory</t>
         </is>
       </c>
-      <c r="I106" s="4" t="inlineStr"/>
-      <c r="J106" s="4" t="inlineStr">
+      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr">
         <is>
           <t>SP-13037</t>
         </is>
       </c>
-      <c r="K106" s="5" t="n">
+      <c r="K106" s="3" t="n">
         <v>45295</v>
       </c>
-      <c r="L106" s="4" t="inlineStr">
+      <c r="L106" s="2" t="inlineStr">
         <is>
           <t>CIN 2-3. Cannot exclude higher grade lesion.</t>
         </is>
       </c>
-      <c r="M106" s="4" t="inlineStr">
+      <c r="M106" s="2" t="inlineStr">
         <is>
           <t>ECC</t>
         </is>
       </c>
-      <c r="N106" s="4" t="inlineStr">
-        <is>
-          <t>HSIL</t>
-        </is>
-      </c>
-      <c r="O106" s="4" t="inlineStr">
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT</t>
+        </is>
+      </c>
+      <c r="O106" s="2" t="inlineStr">
         <is>
           <t>HSIL (CIN3)</t>
         </is>
       </c>
-      <c r="P106" s="4" t="inlineStr">
-        <is>
-          <t>HSIL</t>
-        </is>
-      </c>
-      <c r="Q106" s="4" t="inlineStr">
+      <c r="P106" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT</t>
+        </is>
+      </c>
+      <c r="Q106" s="2" t="inlineStr">
         <is>
           <t>HSIL (CIN3)</t>
         </is>
       </c>
-      <c r="R106" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="S106" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="T106" s="4" t="inlineStr">
-        <is>
-          <t>concordant</t>
-        </is>
-      </c>
-      <c r="U106" s="4" t="inlineStr">
-        <is>
-          <t>exact_agreement</t>
-        </is>
-      </c>
-      <c r="V106" s="4" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="W106" s="4" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="X106" s="4" t="inlineStr">
-        <is>
-          <t>HSIL→HSIL (CIN3)</t>
-        </is>
-      </c>
-      <c r="Y106" s="4" t="b">
+      <c r="R106" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S106" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T106" s="2" t="inlineStr">
+        <is>
+          <t>minor_discordant</t>
+        </is>
+      </c>
+      <c r="U106" s="2" t="inlineStr">
+        <is>
+          <t>minor_overcall</t>
+        </is>
+      </c>
+      <c r="V106" s="2" t="inlineStr">
+        <is>
+          <t>overcall</t>
+        </is>
+      </c>
+      <c r="W106" s="2" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="X106" s="2" t="inlineStr">
+        <is>
+          <t>MALIGNANT→HSIL (CIN3)</t>
+        </is>
+      </c>
+      <c r="Y106" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -12861,7 +12861,7 @@
       </c>
       <c r="O112" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="P112" s="6" t="inlineStr">
@@ -12871,7 +12871,7 @@
       </c>
       <c r="Q112" s="6" t="inlineStr">
         <is>
-          <t>HSIL (CIN3)</t>
+          <t>HSIL (CIN2)</t>
         </is>
       </c>
       <c r="R112" s="6" t="b">
@@ -12902,7 +12902,7 @@
       </c>
       <c r="X112" s="6" t="inlineStr">
         <is>
-          <t>NILM→HSIL (CIN3)</t>
+          <t>NILM→HSIL (CIN2)</t>
         </is>
       </c>
       <c r="Y112" s="6" t="b">
@@ -15056,10 +15056,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" t="n">
-        <v>39.23</v>
+        <v>40.77</v>
       </c>
     </row>
     <row r="3">
@@ -15069,10 +15069,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" t="n">
-        <v>32.31</v>
+        <v>31.54</v>
       </c>
     </row>
     <row r="4">
@@ -15082,10 +15082,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C4" t="n">
-        <v>28.46</v>
+        <v>27.69</v>
       </c>
     </row>
   </sheetData>
@@ -15126,10 +15126,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C2" t="n">
-        <v>28.46</v>
+        <v>27.69</v>
       </c>
     </row>
     <row r="3">
@@ -15139,10 +15139,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C3" t="n">
-        <v>23.85</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="4">
@@ -15165,10 +15165,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" t="n">
-        <v>12.31</v>
+        <v>13.08</v>
       </c>
     </row>
     <row r="6">
@@ -15178,10 +15178,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" t="n">
-        <v>11.54</v>
+        <v>10.77</v>
       </c>
     </row>
     <row r="7">
@@ -15235,10 +15235,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C2" t="n">
-        <v>44.62</v>
+        <v>45.38</v>
       </c>
     </row>
     <row r="3">
@@ -15248,10 +15248,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" t="n">
-        <v>28.46</v>
+        <v>27.69</v>
       </c>
     </row>
     <row r="4">
@@ -15318,10 +15318,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" t="n">
-        <v>39.23</v>
+        <v>40.77</v>
       </c>
     </row>
     <row r="3">
@@ -15331,10 +15331,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" t="n">
-        <v>32.31</v>
+        <v>31.54</v>
       </c>
     </row>
     <row r="4">
@@ -15344,10 +15344,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C4" t="n">
-        <v>28.46</v>
+        <v>27.69</v>
       </c>
     </row>
   </sheetData>
@@ -15361,7 +15361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15420,7 +15420,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>2</v>
@@ -15429,20 +15429,20 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>AGC-ECX/EMC NEO</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -15454,20 +15454,20 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>AIS</t>
         </is>
       </c>
       <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
         <v>1</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -15479,148 +15479,148 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>AIS</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
         <v>3</v>
       </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>ASC-US</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="n">
         <v>2</v>
       </c>
-      <c r="E7" t="n">
-        <v>4</v>
-      </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="n">
         <v>7</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>4</v>
       </c>
-      <c r="E8" t="n">
-        <v>5</v>
-      </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
         <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="n">
         <v>4</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
@@ -15629,50 +15629,25 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>OTHER (EMC45)</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -15709,7 +15684,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>34.62</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="3">
@@ -15719,7 +15694,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38.46</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="4">
@@ -15729,7 +15704,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26.92</v>
+        <v>27.27</v>
       </c>
     </row>
     <row r="5">
@@ -15749,7 +15724,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34.62</v>
+        <v>36.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>